<commit_message>
Add final Windows PostgreSQL business check
</commit_message>
<xml_diff>
--- a/任务规格转化.xlsx
+++ b/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Rd8a92664a6cc4a55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R440623e5e49641ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -346,7 +346,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>通知平台的保留策略、分区库存、租户月度容量和脱敏事件样本</x:v>
+        <x:v>本次业务输入包含通知平台保留策略、分区库存、租户月度容量和通知事件记录</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
@@ -383,57 +383,89 @@
     </x:row>
     <x:row r="10" ht="33" customHeight="1">
       <x:c r="A10" s="5" t="str">
+        <x:v>业务目标</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="str">
+        <x:v>在低峰窗口收缩通知事件热分区，并让活动分区的新部分索引完整接管旧索引</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
+      <x:c r="A11" s="5" t="str">
+        <x:v>交付要求</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>交付完成SQL、分区行动计划、索引交接清单、租户保留审计和变更交接记录，数据库对象与共享字段跨文件一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="33" customHeight="1">
+      <x:c r="A12" s="5" t="str">
+        <x:v>软件步骤</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="str">
+        <x:v>用psql原生载入业务输入；查询catalog；并发处理分区与索引；导出数据库查询结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="33" customHeight="1">
+      <x:c r="A13" s="5" t="str">
         <x:v>业务角色</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B13" s="5" t="str">
         <x:v>数据可靠性团队实施变更，容量值班、DBA、合规人员和变更负责人分别消费交付</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="33" customHeight="1">
-      <x:c r="A11" s="5" t="str">
-        <x:v>分区规则</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="str">
-        <x:v>先确认默认分区为空，再临时脱离默认分区，逐条并发脱离过期月，最后按DEFAULT回挂</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="48" customHeight="1">
-      <x:c r="A12" s="5" t="str">
-        <x:v>索引规则</x:v>
-      </x:c>
-      <x:c r="B12" s="5" t="str">
-        <x:v>键序和状态范围来自策略，活动子索引并发创建，父索引在ONLY父表建立，子索引全部附着后再处置旧索引</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="48" customHeight="1">
-      <x:c r="A13" s="5" t="str">
-        <x:v>数据来源</x:v>
-      </x:c>
-      <x:c r="B13" s="5" t="str">
-        <x:v>分区范围与旧索引身份来自库存，容量来自两份快照，实际对象状态来自PostgreSQL catalog</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="33" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>分区规则</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>process.ps1正常结束，五项交付可读，分区、索引、容量与窗口字段跨文件一致</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="33" customHeight="1">
+        <x:v>先确认默认分区为空，再临时脱离默认分区，逐条并发脱离过期月，最后按DEFAULT回挂</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>索引规则</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>库存覆盖、保留边界、父子关系、索引定义、旧索引处置、租户汇总、窗口信息和文件行数</x:v>
+        <x:v>键序和状态范围来自策略，活动子索引并发创建，父索引在ONLY父表建立，子索引全部附着后再处置旧索引</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="5" t="str">
+        <x:v>数据来源</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="str">
+        <x:v>分区范围与旧索引身份来自库存，容量来自两份快照，实际对象状态来自PostgreSQL catalog</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
+      <x:c r="A17" s="5" t="str">
+        <x:v>实现边界</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="str">
+        <x:v>保留范围、索引列、状态集合和归档路径由策略与库存驱动；分区父子关系、索引定义及有效性来自当前PostgreSQL catalog</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="33" customHeight="1">
+      <x:c r="A18" s="5" t="str">
+        <x:v>完成条件</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>process.ps1正常结束，五项交付可读，分区、索引、容量与窗口字段跨文件一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="33" customHeight="1">
+      <x:c r="A19" s="5" t="str">
+        <x:v>可验证点</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="str">
+        <x:v>库存覆盖、保留边界、父子关系、索引定义、旧索引处置、租户汇总、窗口信息和文件行数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="48" customHeight="1">
+      <x:c r="A20" s="5" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="str">
+      <x:c r="B20" s="5" t="str">
         <x:v>SQL排版、注释风格、CSV行序与行尾、JSON键序和PostgreSQL17.x或18.x补丁版本</x:v>
       </x:c>
     </x:row>

</xml_diff>